<commit_message>
Add configurable dev release logger
</commit_message>
<xml_diff>
--- a/docs/design/蛋仔--大富翁--黑市表.xlsx
+++ b/docs/design/蛋仔--大富翁--黑市表.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29426"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29628"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Administrator\Desktop\eggitor\1_开发中\大富翁\monopoly\design\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Lzx_8\Desktop\eggitor\1_开发中\大富翁\策划案\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5810EA8F-7B44-4848-B781-FC103C7B7A5B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C1417645-4073-4C74-B3F2-59C87FEDA277}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -28,7 +28,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="107" uniqueCount="45">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="125" uniqueCount="52">
   <si>
     <t>字符串</t>
     <phoneticPr fontId="1" type="noConversion"/>
@@ -207,6 +207,34 @@
   </si>
   <si>
     <t>全局限量</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>小猪佩奇</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>小猪乔治</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>海绵宝宝</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>派大星</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>奶龙</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>水豚嘟嘟</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>皮肤商店</t>
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
 </sst>
@@ -214,17 +242,17 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="2" x14ac:knownFonts="1">
+  <fonts count="2">
     <font>
       <sz val="11"/>
       <color theme="1"/>
-      <name val="等线"/>
+      <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
     </font>
     <font>
       <sz val="9"/>
-      <name val="等线"/>
+      <name val="Calibri"/>
       <family val="3"/>
       <charset val="134"/>
       <scheme val="minor"/>
@@ -555,15 +583,15 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:G33"/>
-  <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.2"/>
+  <dimension ref="A1:G39"/>
+  <sheetFormatPr defaultRowHeight="15"/>
   <cols>
-    <col min="3" max="3" width="11.125" customWidth="1"/>
-    <col min="5" max="6" width="11.875" customWidth="1"/>
-    <col min="7" max="7" width="10.5" customWidth="1"/>
+    <col min="3" max="3" width="11.140625" customWidth="1"/>
+    <col min="5" max="6" width="11.85546875" customWidth="1"/>
+    <col min="7" max="7" width="10.42578125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:7">
       <c r="A1" s="1" t="s">
         <v>43</v>
       </c>
@@ -586,7 +614,7 @@
         <v>44</v>
       </c>
     </row>
-    <row r="2" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="2" spans="1:7">
       <c r="A2" s="1" t="s">
         <v>1</v>
       </c>
@@ -609,7 +637,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="3" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="3" spans="1:7">
       <c r="A3" s="1">
         <v>1</v>
       </c>
@@ -632,7 +660,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="4" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="4" spans="1:7">
       <c r="A4" s="1">
         <v>2</v>
       </c>
@@ -655,7 +683,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="5" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="5" spans="1:7">
       <c r="A5" s="1">
         <v>3</v>
       </c>
@@ -678,7 +706,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="6" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="6" spans="1:7">
       <c r="A6" s="1">
         <v>4</v>
       </c>
@@ -701,7 +729,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="7" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="7" spans="1:7">
       <c r="A7" s="1">
         <v>5</v>
       </c>
@@ -724,7 +752,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="8" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="8" spans="1:7">
       <c r="A8" s="1">
         <v>6</v>
       </c>
@@ -747,7 +775,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="9" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="9" spans="1:7">
       <c r="A9" s="1">
         <v>7</v>
       </c>
@@ -770,7 +798,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="10" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="10" spans="1:7">
       <c r="A10" s="1">
         <v>8</v>
       </c>
@@ -793,7 +821,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="11" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="11" spans="1:7">
       <c r="A11" s="1">
         <v>9</v>
       </c>
@@ -816,7 +844,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="12" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="12" spans="1:7">
       <c r="A12" s="1">
         <v>10</v>
       </c>
@@ -839,7 +867,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="13" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="13" spans="1:7">
       <c r="A13" s="1">
         <v>11</v>
       </c>
@@ -862,7 +890,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="14" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="14" spans="1:7">
       <c r="A14" s="1">
         <v>12</v>
       </c>
@@ -885,7 +913,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="15" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="15" spans="1:7">
       <c r="A15" s="1">
         <v>13</v>
       </c>
@@ -908,7 +936,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="16" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="16" spans="1:7">
       <c r="A16" s="1">
         <v>14</v>
       </c>
@@ -931,7 +959,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="17" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="17" spans="1:7">
       <c r="A17" s="1">
         <v>15</v>
       </c>
@@ -954,7 +982,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="18" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="18" spans="1:7">
       <c r="A18" s="1">
         <v>16</v>
       </c>
@@ -977,7 +1005,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="19" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="19" spans="1:7">
       <c r="A19" s="1">
         <v>17</v>
       </c>
@@ -1000,7 +1028,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="20" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="20" spans="1:7">
       <c r="A20" s="1">
         <v>18</v>
       </c>
@@ -1023,7 +1051,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="21" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="21" spans="1:7">
       <c r="A21" s="1">
         <v>19</v>
       </c>
@@ -1046,87 +1074,87 @@
         <v>5</v>
       </c>
     </row>
-    <row r="22" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="22" spans="1:7">
       <c r="A22" s="1">
         <v>20</v>
       </c>
-      <c r="B22" s="2">
-        <v>4001</v>
+      <c r="B22" s="1">
+        <v>5001</v>
       </c>
       <c r="C22" s="2" t="s">
-        <v>9</v>
+        <v>45</v>
       </c>
       <c r="D22" s="2" t="s">
-        <v>42</v>
+        <v>51</v>
       </c>
       <c r="E22" s="2" t="s">
         <v>4</v>
       </c>
       <c r="F22" s="2">
-        <v>98</v>
+        <v>198</v>
       </c>
       <c r="G22" s="2">
         <v>1</v>
       </c>
     </row>
-    <row r="23" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="23" spans="1:7">
       <c r="A23" s="1">
         <v>21</v>
       </c>
-      <c r="B23" s="2">
-        <v>4002</v>
+      <c r="B23" s="1">
+        <v>5002</v>
       </c>
       <c r="C23" s="2" t="s">
-        <v>10</v>
+        <v>46</v>
       </c>
       <c r="D23" s="2" t="s">
-        <v>42</v>
+        <v>51</v>
       </c>
       <c r="E23" s="2" t="s">
         <v>4</v>
       </c>
       <c r="F23" s="2">
-        <v>98</v>
+        <v>198</v>
       </c>
       <c r="G23" s="2">
         <v>1</v>
       </c>
     </row>
-    <row r="24" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="24" spans="1:7">
       <c r="A24" s="1">
         <v>22</v>
       </c>
-      <c r="B24" s="2">
-        <v>4003</v>
+      <c r="B24" s="1">
+        <v>5003</v>
       </c>
       <c r="C24" s="2" t="s">
-        <v>11</v>
+        <v>47</v>
       </c>
       <c r="D24" s="2" t="s">
-        <v>42</v>
+        <v>51</v>
       </c>
       <c r="E24" s="2" t="s">
         <v>4</v>
       </c>
       <c r="F24" s="2">
-        <v>98</v>
+        <v>198</v>
       </c>
       <c r="G24" s="2">
         <v>1</v>
       </c>
     </row>
-    <row r="25" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="25" spans="1:7">
       <c r="A25" s="1">
         <v>23</v>
       </c>
-      <c r="B25" s="2">
-        <v>4004</v>
+      <c r="B25" s="1">
+        <v>5004</v>
       </c>
       <c r="C25" s="2" t="s">
-        <v>12</v>
+        <v>48</v>
       </c>
       <c r="D25" s="2" t="s">
-        <v>42</v>
+        <v>51</v>
       </c>
       <c r="E25" s="2" t="s">
         <v>4</v>
@@ -1138,18 +1166,18 @@
         <v>1</v>
       </c>
     </row>
-    <row r="26" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="26" spans="1:7">
       <c r="A26" s="1">
         <v>24</v>
       </c>
-      <c r="B26" s="2">
-        <v>4005</v>
+      <c r="B26" s="1">
+        <v>5005</v>
       </c>
       <c r="C26" s="2" t="s">
-        <v>13</v>
+        <v>49</v>
       </c>
       <c r="D26" s="2" t="s">
-        <v>42</v>
+        <v>51</v>
       </c>
       <c r="E26" s="2" t="s">
         <v>4</v>
@@ -1161,18 +1189,18 @@
         <v>1</v>
       </c>
     </row>
-    <row r="27" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="27" spans="1:7">
       <c r="A27" s="1">
         <v>25</v>
       </c>
-      <c r="B27" s="2">
-        <v>4006</v>
+      <c r="B27" s="1">
+        <v>5006</v>
       </c>
       <c r="C27" s="2" t="s">
-        <v>14</v>
+        <v>50</v>
       </c>
       <c r="D27" s="2" t="s">
-        <v>42</v>
+        <v>51</v>
       </c>
       <c r="E27" s="2" t="s">
         <v>4</v>
@@ -1184,15 +1212,15 @@
         <v>1</v>
       </c>
     </row>
-    <row r="28" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="28" spans="1:7">
       <c r="A28" s="1">
-        <v>26</v>
+        <v>-1</v>
       </c>
       <c r="B28" s="2">
-        <v>4007</v>
+        <v>4001</v>
       </c>
       <c r="C28" s="2" t="s">
-        <v>15</v>
+        <v>9</v>
       </c>
       <c r="D28" s="2" t="s">
         <v>42</v>
@@ -1201,21 +1229,21 @@
         <v>4</v>
       </c>
       <c r="F28" s="2">
-        <v>998</v>
+        <v>98</v>
       </c>
       <c r="G28" s="2">
         <v>1</v>
       </c>
     </row>
-    <row r="29" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="29" spans="1:7">
       <c r="A29" s="1">
-        <v>27</v>
+        <v>-1</v>
       </c>
       <c r="B29" s="2">
-        <v>4008</v>
+        <v>4002</v>
       </c>
       <c r="C29" s="2" t="s">
-        <v>16</v>
+        <v>10</v>
       </c>
       <c r="D29" s="2" t="s">
         <v>42</v>
@@ -1224,21 +1252,21 @@
         <v>4</v>
       </c>
       <c r="F29" s="2">
-        <v>998</v>
+        <v>98</v>
       </c>
       <c r="G29" s="2">
         <v>1</v>
       </c>
     </row>
-    <row r="30" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="30" spans="1:7">
       <c r="A30" s="1">
-        <v>28</v>
+        <v>-1</v>
       </c>
       <c r="B30" s="2">
-        <v>4009</v>
+        <v>4003</v>
       </c>
       <c r="C30" s="2" t="s">
-        <v>17</v>
+        <v>11</v>
       </c>
       <c r="D30" s="2" t="s">
         <v>42</v>
@@ -1247,21 +1275,21 @@
         <v>4</v>
       </c>
       <c r="F30" s="2">
-        <v>998</v>
+        <v>98</v>
       </c>
       <c r="G30" s="2">
         <v>1</v>
       </c>
     </row>
-    <row r="31" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="31" spans="1:7">
       <c r="A31" s="1">
-        <v>29</v>
+        <v>-1</v>
       </c>
       <c r="B31" s="2">
-        <v>4010</v>
+        <v>4004</v>
       </c>
       <c r="C31" s="2" t="s">
-        <v>18</v>
+        <v>12</v>
       </c>
       <c r="D31" s="2" t="s">
         <v>42</v>
@@ -1270,21 +1298,21 @@
         <v>4</v>
       </c>
       <c r="F31" s="2">
-        <v>1980</v>
+        <v>198</v>
       </c>
       <c r="G31" s="2">
         <v>1</v>
       </c>
     </row>
-    <row r="32" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="32" spans="1:7">
       <c r="A32" s="1">
-        <v>30</v>
+        <v>-1</v>
       </c>
       <c r="B32" s="2">
-        <v>4011</v>
+        <v>4005</v>
       </c>
       <c r="C32" s="2" t="s">
-        <v>19</v>
+        <v>13</v>
       </c>
       <c r="D32" s="2" t="s">
         <v>42</v>
@@ -1293,21 +1321,21 @@
         <v>4</v>
       </c>
       <c r="F32" s="2">
-        <v>1980</v>
+        <v>198</v>
       </c>
       <c r="G32" s="2">
         <v>1</v>
       </c>
     </row>
-    <row r="33" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="33" spans="1:7">
       <c r="A33" s="1">
-        <v>31</v>
+        <v>-1</v>
       </c>
       <c r="B33" s="2">
-        <v>4012</v>
+        <v>4006</v>
       </c>
       <c r="C33" s="2" t="s">
-        <v>20</v>
+        <v>14</v>
       </c>
       <c r="D33" s="2" t="s">
         <v>42</v>
@@ -1316,9 +1344,147 @@
         <v>4</v>
       </c>
       <c r="F33" s="2">
+        <v>198</v>
+      </c>
+      <c r="G33" s="2">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="34" spans="1:7">
+      <c r="A34" s="1">
+        <v>-1</v>
+      </c>
+      <c r="B34" s="2">
+        <v>4007</v>
+      </c>
+      <c r="C34" s="2" t="s">
+        <v>15</v>
+      </c>
+      <c r="D34" s="2" t="s">
+        <v>42</v>
+      </c>
+      <c r="E34" s="2" t="s">
+        <v>4</v>
+      </c>
+      <c r="F34" s="2">
+        <v>998</v>
+      </c>
+      <c r="G34" s="2">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="35" spans="1:7">
+      <c r="A35" s="1">
+        <v>-1</v>
+      </c>
+      <c r="B35" s="2">
+        <v>4008</v>
+      </c>
+      <c r="C35" s="2" t="s">
+        <v>16</v>
+      </c>
+      <c r="D35" s="2" t="s">
+        <v>42</v>
+      </c>
+      <c r="E35" s="2" t="s">
+        <v>4</v>
+      </c>
+      <c r="F35" s="2">
+        <v>998</v>
+      </c>
+      <c r="G35" s="2">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="36" spans="1:7">
+      <c r="A36" s="1">
+        <v>-1</v>
+      </c>
+      <c r="B36" s="2">
+        <v>4009</v>
+      </c>
+      <c r="C36" s="2" t="s">
+        <v>17</v>
+      </c>
+      <c r="D36" s="2" t="s">
+        <v>42</v>
+      </c>
+      <c r="E36" s="2" t="s">
+        <v>4</v>
+      </c>
+      <c r="F36" s="2">
+        <v>998</v>
+      </c>
+      <c r="G36" s="2">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="37" spans="1:7">
+      <c r="A37" s="1">
+        <v>-1</v>
+      </c>
+      <c r="B37" s="2">
+        <v>4010</v>
+      </c>
+      <c r="C37" s="2" t="s">
+        <v>18</v>
+      </c>
+      <c r="D37" s="2" t="s">
+        <v>42</v>
+      </c>
+      <c r="E37" s="2" t="s">
+        <v>4</v>
+      </c>
+      <c r="F37" s="2">
         <v>1980</v>
       </c>
-      <c r="G33" s="2">
+      <c r="G37" s="2">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="38" spans="1:7">
+      <c r="A38" s="1">
+        <v>-1</v>
+      </c>
+      <c r="B38" s="2">
+        <v>4011</v>
+      </c>
+      <c r="C38" s="2" t="s">
+        <v>19</v>
+      </c>
+      <c r="D38" s="2" t="s">
+        <v>42</v>
+      </c>
+      <c r="E38" s="2" t="s">
+        <v>4</v>
+      </c>
+      <c r="F38" s="2">
+        <v>1980</v>
+      </c>
+      <c r="G38" s="2">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="39" spans="1:7">
+      <c r="A39" s="1">
+        <v>-1</v>
+      </c>
+      <c r="B39" s="2">
+        <v>4012</v>
+      </c>
+      <c r="C39" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="D39" s="2" t="s">
+        <v>42</v>
+      </c>
+      <c r="E39" s="2" t="s">
+        <v>4</v>
+      </c>
+      <c r="F39" s="2">
+        <v>1980</v>
+      </c>
+      <c r="G39" s="2">
         <v>1</v>
       </c>
     </row>

</xml_diff>